<commit_message>
sorted in alpha order
</commit_message>
<xml_diff>
--- a/Molecular_data/Lenti_seqs.xlsx
+++ b/Molecular_data/Lenti_seqs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moba692/GitHub/masafumiPhD/Lentibulariaceae/Molecular_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moba692/GitHub/CPs/Molecular_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29BFA1AC-74C1-0E4D-AC6B-719541A39042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F53219-55AC-474A-897E-833E602AAB1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2480" yWindow="680" windowWidth="29220" windowHeight="18960" activeTab="1" xr2:uid="{2CC7BAB4-51AF-4B46-92E5-E6D61800B7D9}"/>
+    <workbookView xWindow="40" yWindow="680" windowWidth="29220" windowHeight="18960" activeTab="2" xr2:uid="{2CC7BAB4-51AF-4B46-92E5-E6D61800B7D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Pinguicula" sheetId="4" r:id="rId1"/>
@@ -4409,7 +4409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4478,9 +4478,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9193,7 +9190,7 @@
     <col min="3" max="3" width="16" style="16" customWidth="1"/>
     <col min="4" max="4" width="29.5" style="21" customWidth="1"/>
     <col min="5" max="5" width="17.1640625" style="16" customWidth="1"/>
-    <col min="6" max="6" width="34" style="31" customWidth="1"/>
+    <col min="6" max="6" width="34" style="14" customWidth="1"/>
     <col min="7" max="7" width="17.83203125" style="16" customWidth="1"/>
     <col min="8" max="8" width="36.83203125" style="14" customWidth="1"/>
     <col min="9" max="9" width="24" style="19" customWidth="1"/>
@@ -9268,7 +9265,7 @@
       <c r="E2" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="31" t="s">
+      <c r="F2" s="14" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="16" t="s">
@@ -9304,7 +9301,7 @@
       <c r="E3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="31" t="s">
+      <c r="F3" s="14" t="s">
         <v>12</v>
       </c>
       <c r="G3" s="16" t="s">
@@ -9340,7 +9337,7 @@
       <c r="E4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G4" s="16" t="s">
@@ -9375,7 +9372,7 @@
       <c r="E5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="14" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="16" t="s">
@@ -9410,7 +9407,7 @@
       <c r="E6" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="14" t="s">
         <v>20</v>
       </c>
       <c r="G6" s="16" t="s">
@@ -9445,7 +9442,7 @@
       <c r="E7" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G7" s="16" t="s">
@@ -9480,7 +9477,7 @@
       <c r="E8" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="14" t="s">
         <v>33</v>
       </c>
       <c r="G8" s="16" t="s">
@@ -9515,7 +9512,7 @@
       <c r="E9" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="14" t="s">
         <v>37</v>
       </c>
       <c r="G9" s="16" t="s">
@@ -10320,7 +10317,7 @@
       <c r="E32" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F32" s="31" t="s">
+      <c r="F32" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G32" s="18" t="s">
@@ -10355,7 +10352,7 @@
       <c r="E33" s="30" t="s">
         <v>1257</v>
       </c>
-      <c r="F33" s="31" t="s">
+      <c r="F33" s="14" t="s">
         <v>1258</v>
       </c>
       <c r="G33" s="18" t="s">
@@ -10390,7 +10387,7 @@
       <c r="E34" s="30" t="s">
         <v>1262</v>
       </c>
-      <c r="F34" s="31" t="s">
+      <c r="F34" s="14" t="s">
         <v>625</v>
       </c>
       <c r="G34" s="18" t="s">
@@ -10425,7 +10422,7 @@
       <c r="E35" s="30" t="s">
         <v>1267</v>
       </c>
-      <c r="F35" s="31" t="s">
+      <c r="F35" s="14" t="s">
         <v>606</v>
       </c>
       <c r="G35" s="18" t="s">
@@ -10460,7 +10457,7 @@
       <c r="E36" s="30" t="s">
         <v>1272</v>
       </c>
-      <c r="F36" s="31" t="s">
+      <c r="F36" s="14" t="s">
         <v>1258</v>
       </c>
       <c r="G36" s="16" t="s">
@@ -10495,7 +10492,7 @@
       <c r="E37" s="30" t="s">
         <v>1277</v>
       </c>
-      <c r="F37" s="31" t="s">
+      <c r="F37" s="14" t="s">
         <v>625</v>
       </c>
       <c r="G37" s="18" t="s">
@@ -10530,7 +10527,7 @@
       <c r="E38" s="30" t="s">
         <v>1278</v>
       </c>
-      <c r="F38" s="31" t="s">
+      <c r="F38" s="14" t="s">
         <v>1258</v>
       </c>
       <c r="G38" s="16" t="s">
@@ -10565,7 +10562,7 @@
       <c r="E39" s="30" t="s">
         <v>1283</v>
       </c>
-      <c r="F39" s="31" t="s">
+      <c r="F39" s="14" t="s">
         <v>1284</v>
       </c>
       <c r="G39" s="18" t="s">
@@ -10600,7 +10597,7 @@
       <c r="E40" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F40" s="31" t="s">
+      <c r="F40" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G40" s="16" t="s">
@@ -10635,7 +10632,7 @@
       <c r="E41" s="30" t="s">
         <v>1291</v>
       </c>
-      <c r="F41" s="31" t="s">
+      <c r="F41" s="14" t="s">
         <v>625</v>
       </c>
       <c r="G41" s="18" t="s">
@@ -10670,7 +10667,7 @@
       <c r="E42" s="30" t="s">
         <v>1296</v>
       </c>
-      <c r="F42" s="31" t="s">
+      <c r="F42" s="14" t="s">
         <v>606</v>
       </c>
       <c r="G42" s="18" t="s">
@@ -10705,7 +10702,7 @@
       <c r="E43" s="30" t="s">
         <v>1301</v>
       </c>
-      <c r="F43" s="31" t="s">
+      <c r="F43" s="14" t="s">
         <v>935</v>
       </c>
       <c r="G43" s="18" t="s">
@@ -10740,7 +10737,7 @@
       <c r="E44" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F44" s="31" t="s">
+      <c r="F44" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G44" s="16" t="s">
@@ -10775,7 +10772,7 @@
       <c r="E45" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F45" s="31" t="s">
+      <c r="F45" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G45" s="16" t="s">
@@ -10810,7 +10807,7 @@
       <c r="E46" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F46" s="31" t="s">
+      <c r="F46" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G46" s="16" t="s">
@@ -10845,7 +10842,7 @@
       <c r="E47" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F47" s="31" t="s">
+      <c r="F47" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G47" s="18" t="s">
@@ -10880,7 +10877,7 @@
       <c r="E48" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F48" s="31" t="s">
+      <c r="F48" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G48" s="16" t="s">
@@ -10915,7 +10912,7 @@
       <c r="E49" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F49" s="31" t="s">
+      <c r="F49" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G49" s="16" t="s">
@@ -10950,7 +10947,7 @@
       <c r="E50" s="30" t="s">
         <v>1319</v>
       </c>
-      <c r="F50" s="31" t="s">
+      <c r="F50" s="14" t="s">
         <v>1320</v>
       </c>
       <c r="G50" s="18" t="s">
@@ -10985,7 +10982,7 @@
       <c r="E51" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F51" s="31" t="s">
+      <c r="F51" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G51" s="16" t="s">
@@ -11020,7 +11017,7 @@
       <c r="E52" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F52" s="31" t="s">
+      <c r="F52" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G52" s="18" t="s">
@@ -11055,7 +11052,7 @@
       <c r="E53" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F53" s="31" t="s">
+      <c r="F53" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G53" s="18" t="s">
@@ -11090,7 +11087,7 @@
       <c r="E54" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F54" s="31" t="s">
+      <c r="F54" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G54" s="18" t="s">
@@ -11125,7 +11122,7 @@
       <c r="E55" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F55" s="31" t="s">
+      <c r="F55" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G55" s="18" t="s">
@@ -11160,7 +11157,7 @@
       <c r="E56" s="30" t="s">
         <v>1345</v>
       </c>
-      <c r="F56" s="31" t="s">
+      <c r="F56" s="14" t="s">
         <v>1258</v>
       </c>
       <c r="G56" s="18" t="s">
@@ -11195,7 +11192,7 @@
       <c r="E57" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F57" s="31" t="s">
+      <c r="F57" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G57" s="18" t="s">
@@ -11230,7 +11227,7 @@
       <c r="E58" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F58" s="31" t="s">
+      <c r="F58" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G58" s="18" t="s">
@@ -11265,7 +11262,7 @@
       <c r="E59" s="30" t="s">
         <v>1359</v>
       </c>
-      <c r="F59" s="31" t="s">
+      <c r="F59" s="14" t="s">
         <v>1360</v>
       </c>
       <c r="G59" s="18" t="s">
@@ -11300,7 +11297,7 @@
       <c r="E60" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F60" s="31" t="s">
+      <c r="F60" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G60" s="16" t="s">
@@ -11335,7 +11332,7 @@
       <c r="E61" s="30" t="s">
         <v>1369</v>
       </c>
-      <c r="F61" s="31" t="s">
+      <c r="F61" s="14" t="s">
         <v>1370</v>
       </c>
       <c r="G61" s="18" t="s">
@@ -11370,7 +11367,7 @@
       <c r="E62" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F62" s="31" t="s">
+      <c r="F62" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G62" s="16" t="s">
@@ -11405,7 +11402,7 @@
       <c r="E63" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F63" s="31" t="s">
+      <c r="F63" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G63" s="18" t="s">
@@ -11440,7 +11437,7 @@
       <c r="E64" s="30" t="s">
         <v>1385</v>
       </c>
-      <c r="F64" s="31" t="s">
+      <c r="F64" s="14" t="s">
         <v>1360</v>
       </c>
       <c r="G64" s="18" t="s">
@@ -11475,7 +11472,7 @@
       <c r="E65" s="30" t="s">
         <v>1389</v>
       </c>
-      <c r="F65" s="31" t="s">
+      <c r="F65" s="14" t="s">
         <v>1390</v>
       </c>
       <c r="G65" s="18" t="s">
@@ -11510,7 +11507,7 @@
       <c r="E66" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F66" s="31" t="s">
+      <c r="F66" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G66" s="16" t="s">
@@ -11545,7 +11542,7 @@
       <c r="E67" s="30" t="s">
         <v>1398</v>
       </c>
-      <c r="F67" s="31" t="s">
+      <c r="F67" s="14" t="s">
         <v>1399</v>
       </c>
       <c r="G67" s="18" t="s">
@@ -11580,7 +11577,7 @@
       <c r="E68" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F68" s="31" t="s">
+      <c r="F68" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G68" s="16" t="s">
@@ -13027,7 +13024,7 @@
       <c r="E158" s="18" t="s">
         <v>496</v>
       </c>
-      <c r="F158" s="31" t="s">
+      <c r="F158" s="14" t="s">
         <v>497</v>
       </c>
       <c r="H158" s="27"/>
@@ -13256,7 +13253,7 @@
       <c r="E168" s="18" t="s">
         <v>538</v>
       </c>
-      <c r="F168" s="31" t="s">
+      <c r="F168" s="14" t="s">
         <v>539</v>
       </c>
       <c r="H168" s="27"/>
@@ -13455,7 +13452,7 @@
       <c r="E177" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F177" s="31" t="s">
+      <c r="F177" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G177" s="18" t="s">
@@ -13487,7 +13484,7 @@
       <c r="E178" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F178" s="31" t="s">
+      <c r="F178" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G178" s="18" t="s">
@@ -13519,7 +13516,7 @@
       <c r="E179" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F179" s="31" t="s">
+      <c r="F179" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G179" s="18" t="s">
@@ -13549,7 +13546,7 @@
       <c r="E180" s="18" t="s">
         <v>605</v>
       </c>
-      <c r="F180" s="31" t="s">
+      <c r="F180" s="14" t="s">
         <v>606</v>
       </c>
       <c r="G180" s="18" t="s">
@@ -13579,7 +13576,7 @@
       <c r="E181" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F181" s="31" t="s">
+      <c r="F181" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G181" s="18" t="s">
@@ -13609,7 +13606,7 @@
       <c r="E182" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F182" s="31" t="s">
+      <c r="F182" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G182" s="18" t="s">
@@ -13641,7 +13638,7 @@
       <c r="E183" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F183" s="31" t="s">
+      <c r="F183" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G183" s="18" t="s">
@@ -13671,7 +13668,7 @@
       <c r="E184" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F184" s="31" t="s">
+      <c r="F184" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G184" s="18" t="s">
@@ -13704,7 +13701,7 @@
       <c r="E185" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F185" s="31" t="s">
+      <c r="F185" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G185" s="18" t="s">
@@ -13736,7 +13733,7 @@
       <c r="E186" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F186" s="31" t="s">
+      <c r="F186" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G186" s="18" t="s">
@@ -13768,7 +13765,7 @@
       <c r="E187" s="18" t="s">
         <v>624</v>
       </c>
-      <c r="F187" s="31" t="s">
+      <c r="F187" s="14" t="s">
         <v>625</v>
       </c>
       <c r="G187" s="18" t="s">
@@ -13800,7 +13797,7 @@
       <c r="E188" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F188" s="31" t="s">
+      <c r="F188" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G188" s="18" t="s">
@@ -13832,7 +13829,7 @@
       <c r="E189" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F189" s="31" t="s">
+      <c r="F189" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G189" s="18" t="s">
@@ -13864,7 +13861,7 @@
       <c r="E190" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F190" s="31" t="s">
+      <c r="F190" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G190" s="18" t="s">
@@ -13896,7 +13893,7 @@
       <c r="E191" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F191" s="31" t="s">
+      <c r="F191" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G191" s="18" t="s">
@@ -13928,7 +13925,7 @@
       <c r="E192" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F192" s="31" t="s">
+      <c r="F192" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G192" s="18" t="s">
@@ -13960,7 +13957,7 @@
       <c r="E193" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F193" s="31" t="s">
+      <c r="F193" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G193" s="18" t="s">
@@ -13992,7 +13989,7 @@
       <c r="E194" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F194" s="31" t="s">
+      <c r="F194" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G194" s="18" t="s">
@@ -14027,7 +14024,7 @@
       <c r="E195" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F195" s="31" t="s">
+      <c r="F195" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G195" s="18" t="s">
@@ -14059,7 +14056,7 @@
       <c r="E196" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F196" s="31" t="s">
+      <c r="F196" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G196" s="18" t="s">
@@ -14091,7 +14088,7 @@
       <c r="E197" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F197" s="31" t="s">
+      <c r="F197" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G197" s="18" t="s">
@@ -14123,7 +14120,7 @@
       <c r="E198" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F198" s="31" t="s">
+      <c r="F198" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G198" s="18" t="s">
@@ -14155,7 +14152,7 @@
       <c r="E199" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F199" s="31" t="s">
+      <c r="F199" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G199" s="18" t="s">
@@ -14187,7 +14184,7 @@
       <c r="E200" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F200" s="31" t="s">
+      <c r="F200" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G200" s="18" t="s">
@@ -14219,7 +14216,7 @@
       <c r="E201" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="F201" s="31" t="s">
+      <c r="F201" s="14" t="s">
         <v>343</v>
       </c>
       <c r="G201" s="18" t="s">

</xml_diff>